<commit_message>
arreglo tema pbg, borro cosas no útiles
</commit_message>
<xml_diff>
--- a/Serie PBG.xlsx
+++ b/Serie PBG.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\UNIVERSIDAD ECONOMÍA\Tercer Año\Proyecto-evolucion-salarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Facultad\Proyecto-evolucion-salarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746A2DB8-8A79-4E13-8BD3-92D6F4161408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C025D463-802B-4327-AD1A-CD0D5F2B98EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evolución PBG MZA" sheetId="14" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId18" roundtripDataChecksum="/dUSXa82hxQOGMb+5WJan/aJb6jPiaBSIQkW1CqgTQI="/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="12">
   <si>
     <t>Año</t>
   </si>
@@ -103,19 +103,27 @@
   <si>
     <t>PBG convertido</t>
   </si>
+  <si>
+    <t>Prueba de como poner la variación entre cambios de monedas</t>
+  </si>
+  <si>
+    <t>PBI a precios de mercadoBase Ferreres (mill. de $ 1993)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.000E+00_)"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="168" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="#,##0\ \ \ \ "/>
+    <numFmt numFmtId="170" formatCode="#,##0\ \ "/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +170,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="62"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="62"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -177,7 +208,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -225,11 +256,116 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="14"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -287,15 +423,55 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal_PBI pk por Sectores final" xfId="1" xr:uid="{01AEF0FB-32A3-424C-9468-ECB2E56EA492}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -539,6 +715,12 @@
       <c r="G1" s="21" t="s">
         <v>9</v>
       </c>
+      <c r="M1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
@@ -563,6 +745,12 @@
         <f>B2/$F$2</f>
         <v>3134300</v>
       </c>
+      <c r="M2" s="42">
+        <v>1969</v>
+      </c>
+      <c r="N2" s="41">
+        <v>152643.77335610622</v>
+      </c>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
@@ -585,6 +773,12 @@
         <f>B3/$F$2</f>
         <v>3344100</v>
       </c>
+      <c r="M3" s="43">
+        <v>1970</v>
+      </c>
+      <c r="N3" s="41">
+        <v>160860.95636173122</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
@@ -606,6 +800,12 @@
       <c r="G4" s="22">
         <f t="shared" ref="G4:G17" si="1">B4/$F$2</f>
         <v>3562599.9999999995</v>
+      </c>
+      <c r="M4" s="42">
+        <v>1971</v>
+      </c>
+      <c r="N4" s="41">
+        <v>166912.60622155317</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -635,8 +835,12 @@
       <c r="J5" s="8"/>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
+      <c r="M5" s="42">
+        <v>1972</v>
+      </c>
+      <c r="N5" s="41">
+        <v>170379.33445085437</v>
+      </c>
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
       <c r="Q5" s="9"/>
@@ -662,6 +866,12 @@
       <c r="G6" s="22">
         <f t="shared" si="1"/>
         <v>4063700</v>
+      </c>
+      <c r="M6" s="42">
+        <v>1973</v>
+      </c>
+      <c r="N6" s="41">
+        <v>176760.97430606186</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -691,8 +901,12 @@
       <c r="J7" s="10"/>
       <c r="K7" s="10"/>
       <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
+      <c r="M7" s="42">
+        <v>1974</v>
+      </c>
+      <c r="N7" s="41">
+        <v>186316.01795022786</v>
+      </c>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -716,6 +930,12 @@
         <f t="shared" si="1"/>
         <v>4040500</v>
       </c>
+      <c r="M8" s="42">
+        <v>1975</v>
+      </c>
+      <c r="N8" s="41">
+        <v>185210.55146568603</v>
+      </c>
     </row>
     <row r="9" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
@@ -738,6 +958,12 @@
         <f t="shared" si="1"/>
         <v>3806300</v>
       </c>
+      <c r="M9" s="42">
+        <v>1976</v>
+      </c>
+      <c r="N9" s="41">
+        <v>185188.55213266029</v>
+      </c>
     </row>
     <row r="10" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
@@ -760,6 +986,16 @@
         <f t="shared" si="1"/>
         <v>4236000</v>
       </c>
+      <c r="I10" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="40"/>
+      <c r="M10" s="42">
+        <v>1977</v>
+      </c>
+      <c r="N10" s="41">
+        <v>197015.02691173065</v>
+      </c>
     </row>
     <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
@@ -778,9 +1014,19 @@
       <c r="E11" s="5">
         <v>6.1350683333333345E-7</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="23">
         <f t="shared" si="1"/>
         <v>4810500</v>
+      </c>
+      <c r="H11" s="26"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="28"/>
+      <c r="M11" s="42">
+        <v>1978</v>
+      </c>
+      <c r="N11" s="41">
+        <v>190666.38605606163</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -800,9 +1046,19 @@
       <c r="E12" s="5">
         <v>1.2317019999999998E-6</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="23">
         <f t="shared" si="1"/>
         <v>4292400</v>
+      </c>
+      <c r="H12" s="29"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="31"/>
+      <c r="M12" s="42">
+        <v>1979</v>
+      </c>
+      <c r="N12" s="41">
+        <v>203891.65176001663</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -822,18 +1078,25 @@
       <c r="E13" s="5">
         <v>2.5185499999999998E-6</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="23">
         <f t="shared" si="1"/>
         <v>3518299.9999999995</v>
       </c>
-      <c r="I13" s="23">
+      <c r="H13" s="29"/>
+      <c r="I13" s="32">
         <v>6485507</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="32">
         <v>7035026</v>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="33">
         <v>7761508</v>
+      </c>
+      <c r="M13" s="43">
+        <v>1980</v>
+      </c>
+      <c r="N13" s="41">
+        <v>207011.43217472488</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -853,21 +1116,28 @@
       <c r="E14" s="5">
         <v>6.6685833333333333E-6</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="23">
         <f t="shared" si="1"/>
         <v>3604300</v>
       </c>
-      <c r="I14">
+      <c r="H14" s="29"/>
+      <c r="I14" s="30">
         <f>I13/I15</f>
         <v>24.984713709506547</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="30">
         <f t="shared" ref="J14:K14" si="2">J13/J15</f>
         <v>25.354277414774263</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="31">
         <f t="shared" si="2"/>
         <v>26.13610358123011</v>
+      </c>
+      <c r="M14" s="42">
+        <v>1981</v>
+      </c>
+      <c r="N14" s="41">
+        <v>195787.08557126726</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -887,18 +1157,25 @@
       <c r="E15" s="5">
         <v>2.9595141666666666E-5</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="23">
         <f t="shared" si="1"/>
         <v>4192599.9999999995</v>
       </c>
-      <c r="I15" s="24">
+      <c r="H15" s="29"/>
+      <c r="I15" s="34">
         <v>259579</v>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="34">
         <v>277469</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="35">
         <v>296965</v>
+      </c>
+      <c r="M15" s="42">
+        <v>1982</v>
+      </c>
+      <c r="N15" s="41">
+        <v>189602.24152446413</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -918,9 +1195,19 @@
       <c r="E16" s="5">
         <v>2.1507783333333334E-4</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="23">
         <f t="shared" si="1"/>
         <v>4044400</v>
+      </c>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="31"/>
+      <c r="M16" s="42">
+        <v>1983</v>
+      </c>
+      <c r="N16" s="41">
+        <v>197400.61051265232</v>
       </c>
     </row>
     <row r="17" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -940,13 +1227,22 @@
       <c r="E17" s="5">
         <v>1.6607925000000001E-3</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="23">
         <f t="shared" si="1"/>
         <v>3846100</v>
       </c>
-      <c r="I17">
+      <c r="H17" s="29"/>
+      <c r="I17" s="30">
         <f>AVERAGE(I14:K14)</f>
         <v>25.491698235170304</v>
+      </c>
+      <c r="J17" s="30"/>
+      <c r="K17" s="31"/>
+      <c r="M17" s="42">
+        <v>1984</v>
+      </c>
+      <c r="N17" s="41">
+        <v>201349.02459711238</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -966,12 +1262,21 @@
       <c r="E18" s="5">
         <v>3.1570041666666667E-3</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="24">
         <v>267608.7</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="29">
         <f>G18*$I$17</f>
         <v>6821800.22550622</v>
+      </c>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="31"/>
+      <c r="M18" s="42">
+        <v>1985</v>
+      </c>
+      <c r="N18" s="41">
+        <v>187351.74596487361</v>
       </c>
     </row>
     <row r="19" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -991,12 +1296,21 @@
       <c r="E19" s="5">
         <v>7.3032416666666657E-3</v>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="24">
         <v>271052</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="29">
         <f t="shared" ref="H19:H22" si="4">G19*$I$17</f>
         <v>6909575.790039381</v>
+      </c>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="31"/>
+      <c r="M19" s="42">
+        <v>1986</v>
+      </c>
+      <c r="N19" s="41">
+        <v>200726.11957615431</v>
       </c>
     </row>
     <row r="20" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1016,12 +1330,21 @@
       <c r="E20" s="13">
         <v>3.2350000000000004E-2</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="24">
         <v>264473</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="29">
         <f t="shared" si="4"/>
         <v>6741865.9073501956</v>
+      </c>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="31"/>
+      <c r="M20" s="42">
+        <v>1987</v>
+      </c>
+      <c r="N20" s="41">
+        <v>205926.37181563661</v>
       </c>
     </row>
     <row r="21" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1041,12 +1364,21 @@
       <c r="E21" s="13">
         <v>1.0285535833333335</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G21" s="24">
         <v>253410</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="29">
         <f t="shared" si="4"/>
         <v>6459851.2497745063</v>
+      </c>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="31"/>
+      <c r="M21" s="42">
+        <v>1988</v>
+      </c>
+      <c r="N21" s="41">
+        <v>202022.16389395422</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1066,12 +1398,21 @@
       <c r="E22" s="14">
         <v>24.828900000000001</v>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="24">
         <v>253627</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="29">
         <f t="shared" si="4"/>
         <v>6465382.9482915383</v>
+      </c>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="31"/>
+      <c r="M22" s="42">
+        <v>1989</v>
+      </c>
+      <c r="N22" s="41">
+        <v>188010.819664468</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1092,10 +1433,19 @@
         <v>67.453100000000006</v>
       </c>
       <c r="F23" s="10"/>
-      <c r="G23" s="15">
+      <c r="G23" s="25">
         <v>6485506.9469233276</v>
       </c>
-      <c r="H23" s="10"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="31"/>
+      <c r="M23" s="43">
+        <v>1990</v>
+      </c>
+      <c r="N23" s="41">
+        <v>184568.76708091571</v>
+      </c>
     </row>
     <row r="24" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
@@ -1114,10 +1464,19 @@
       <c r="E24" s="14">
         <v>84.248900000000006</v>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="25">
         <v>7035025.5867938362</v>
       </c>
-      <c r="H24" s="10"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="31"/>
+      <c r="M24" s="42">
+        <v>1991</v>
+      </c>
+      <c r="N24" s="41">
+        <v>204093.82543139864</v>
+      </c>
     </row>
     <row r="25" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
@@ -1136,10 +1495,19 @@
       <c r="E25" s="14">
         <v>93.188999999999993</v>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="25">
         <v>7761508.2247009035</v>
       </c>
-      <c r="H25" s="10"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="39"/>
+      <c r="M25" s="42">
+        <v>1992</v>
+      </c>
+      <c r="N25" s="41">
+        <v>223701.26799433088</v>
+      </c>
     </row>
     <row r="26" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
@@ -1167,8 +1535,12 @@
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
       <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
+      <c r="M26" s="42">
+        <v>1993</v>
+      </c>
+      <c r="N26" s="41">
+        <v>236504.9802315725</v>
+      </c>
       <c r="O26" s="17"/>
       <c r="P26" s="17"/>
       <c r="Q26" s="17"/>
@@ -1199,6 +1571,12 @@
       <c r="G27" s="15">
         <v>7908811.3856461942</v>
       </c>
+      <c r="M27" s="42">
+        <v>1994</v>
+      </c>
+      <c r="N27" s="41">
+        <v>250307.88553631518</v>
+      </c>
     </row>
     <row r="28" spans="1:23" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
@@ -1220,6 +1598,12 @@
       <c r="G28" s="15">
         <v>8135361.8772270568</v>
       </c>
+      <c r="M28" s="42">
+        <v>1995</v>
+      </c>
+      <c r="N28" s="41">
+        <v>243186.10151946038</v>
+      </c>
     </row>
     <row r="29" spans="1:23" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
@@ -1241,6 +1625,12 @@
       <c r="G29" s="15">
         <v>8905959.4449048098</v>
       </c>
+      <c r="M29" s="42">
+        <v>1996</v>
+      </c>
+      <c r="N29" s="41">
+        <v>256626.24305584718</v>
+      </c>
     </row>
     <row r="30" spans="1:23" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
@@ -1262,6 +1652,12 @@
       <c r="G30" s="15">
         <v>9488295.9322833791</v>
       </c>
+      <c r="M30" s="42">
+        <v>1997</v>
+      </c>
+      <c r="N30" s="41">
+        <v>277441.31762238021</v>
+      </c>
     </row>
     <row r="31" spans="1:23" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
@@ -1283,6 +1679,12 @@
       <c r="G31" s="15">
         <v>9252615.1693661101</v>
       </c>
+      <c r="M31" s="42">
+        <v>1998</v>
+      </c>
+      <c r="N31" s="41">
+        <v>288122.8046077239</v>
+      </c>
     </row>
     <row r="32" spans="1:23" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
@@ -1304,6 +1706,12 @@
       <c r="G32" s="15">
         <v>9002038.4513383135</v>
       </c>
+      <c r="M32" s="42">
+        <v>1999</v>
+      </c>
+      <c r="N32" s="41">
+        <v>278369.01387171785</v>
+      </c>
     </row>
     <row r="33" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
@@ -1325,6 +1733,12 @@
       <c r="G33" s="15">
         <v>8322993.4966704417</v>
       </c>
+      <c r="M33" s="43">
+        <v>2000</v>
+      </c>
+      <c r="N33" s="41">
+        <v>276172.18535265006</v>
+      </c>
     </row>
     <row r="34" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
@@ -1346,6 +1760,12 @@
       <c r="G34" s="15">
         <v>7772198.0394271128</v>
       </c>
+      <c r="M34" s="42">
+        <v>2001</v>
+      </c>
+      <c r="N34" s="41">
+        <v>263995.67436681729</v>
+      </c>
     </row>
     <row r="35" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
@@ -1367,6 +1787,12 @@
       <c r="G35" s="15">
         <v>9339929.5945354141</v>
       </c>
+      <c r="M35" s="42">
+        <v>2002</v>
+      </c>
+      <c r="N35" s="41">
+        <v>235234.59675290697</v>
+      </c>
     </row>
     <row r="36" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
@@ -1388,6 +1814,12 @@
       <c r="G36" s="19">
         <v>10874929.097083896</v>
       </c>
+      <c r="M36" s="42">
+        <v>2003</v>
+      </c>
+      <c r="N36" s="41">
+        <v>256022.46524751041</v>
+      </c>
     </row>
     <row r="37" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
@@ -1408,6 +1840,12 @@
       </c>
       <c r="G37" s="19">
         <v>11380763.411127962</v>
+      </c>
+      <c r="M37" s="42">
+        <v>2004</v>
+      </c>
+      <c r="N37" s="41">
+        <v>279020</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
@@ -1562,8 +2000,6 @@
       <c r="J44" s="17"/>
       <c r="K44" s="17"/>
       <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
       <c r="O44" s="17"/>
       <c r="P44" s="17"/>
       <c r="Q44" s="17"/>
@@ -1605,6 +2041,8 @@
       <c r="G45" s="19">
         <v>14211513.62051825</v>
       </c>
+      <c r="M45" s="17"/>
+      <c r="N45" s="17"/>
     </row>
     <row r="46" spans="1:24" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
@@ -1819,6 +2257,9 @@
       <c r="O65" s="17"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I10:J10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>